<commit_message>
Added initial smart questions for review
</commit_message>
<xml_diff>
--- a/midterm/SMART Question Proposals.xlsx
+++ b/midterm/SMART Question Proposals.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/225622b72ce7f783/Documents/GWU/Semester 1/DATS 6101 - Introduction to Data Science/Mid Term Project/team_galileo/midterm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venka\OneDrive\Desktop\Class\6101\Assignments\Midterm project\team_galileo\midterm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{732FCDD9-9275-4B2B-A9D2-1B363CCD3E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8735CA-FB81-470F-85DE-BB06714E8C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">Please include the proposals under your name </t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t xml:space="preserve">SMART Question Proposals </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is there an optimal combination of workout duration, intensity, and sleep hours for maximizing calorie burn while minimizing post-workout fatigue? </t>
+  </si>
+  <si>
+    <t>Is there a link between poor sleep (fewer hours and higher resting heart rate) and increased feelings of fatigue or stress after workouts?</t>
+  </si>
+  <si>
+    <t>Can consistent exercise (tracked by workout type, duration, and frequency) predict improvements in mood after workouts over time?</t>
+  </si>
+  <si>
+    <t>Do users with higher body fat percentages experience greater mood improvements after high-intensity workouts compared to low-intensity sessions?</t>
   </si>
 </sst>
 </file>
@@ -80,12 +92,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -100,10 +118,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,27 +461,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2B683-EEB2-4C59-A502-E3C117712EB0}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" customWidth="1"/>
+    <col min="1" max="1" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.19921875" customWidth="1"/>
+    <col min="3" max="3" width="45.73046875" customWidth="1"/>
+    <col min="4" max="4" width="11.86328125" customWidth="1"/>
+    <col min="5" max="5" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -468,11 +491,31 @@
       <c r="C4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="C8" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Transposed the table and added ranking columns
</commit_message>
<xml_diff>
--- a/midterm/SMART Question Proposals.xlsx
+++ b/midterm/SMART Question Proposals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venka\OneDrive\Desktop\Class\6101\Assignments\Midterm project\team_galileo\midterm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisgamo\Documents\GitHub\team_galileo\midterm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8735CA-FB81-470F-85DE-BB06714E8C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3516DF-7292-4117-A3F4-32BC3B380EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
+    <workbookView xWindow="-38510" yWindow="-3370" windowWidth="38620" windowHeight="21220" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t xml:space="preserve">Please include the proposals under your name </t>
   </si>
@@ -69,13 +67,22 @@
   </si>
   <si>
     <t>Do users with higher body fat percentages experience greater mood improvements after high-intensity workouts compared to low-intensity sessions?</t>
+  </si>
+  <si>
+    <t>Ranking</t>
+  </si>
+  <si>
+    <t>Contributor</t>
+  </si>
+  <si>
+    <t>Question</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,7 +99,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -102,6 +109,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -118,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -126,6 +139,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -461,64 +483,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2B683-EEB2-4C59-A502-E3C117712EB0}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.19921875" customWidth="1"/>
-    <col min="3" max="3" width="45.73046875" customWidth="1"/>
-    <col min="4" max="4" width="11.86328125" customWidth="1"/>
-    <col min="5" max="5" width="13.796875" customWidth="1"/>
+    <col min="1" max="1" width="12.75" customWidth="1"/>
+    <col min="2" max="2" width="34.58203125" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row r="3" spans="1:7">
+      <c r="C3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="1:7">
+      <c r="A5" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="56">
+      <c r="A7" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="C6" s="2" t="s">
+    <row r="8" spans="1:7" ht="56">
+      <c r="A8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="C7" s="3" t="s">
+    <row r="9" spans="1:7" ht="56">
+      <c r="A9" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="C8" s="2" t="s">
+    <row r="10" spans="1:7" ht="70">
+      <c r="A10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="5" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:G3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated dmart ques in xl sheet
</commit_message>
<xml_diff>
--- a/midterm/SMART Question Proposals.xlsx
+++ b/midterm/SMART Question Proposals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MANOJ\Documents\GitHub\team_galileo\midterm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09894054-A81D-4938-9ECA-E0BE660F8E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C658F3BD-3BDD-4C49-A2CE-43B61B603F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
   </bookViews>
@@ -107,7 +107,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -599,7 +599,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Update SMART Question Proposals.xlsx
Added my proposals
</commit_message>
<xml_diff>
--- a/midterm/SMART Question Proposals.xlsx
+++ b/midterm/SMART Question Proposals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisgamo\Documents\GitHub\team_galileo\midterm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/225622b72ce7f783/Documents/GWU/Semester 1/DATS 6101 - Introduction to Data Science/Mid Term Project/team_galileo/midterm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3516DF-7292-4117-A3F4-32BC3B380EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{FF3516DF-7292-4117-A3F4-32BC3B380EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6864B3C-B5B6-4B44-84E3-A2ADA305C908}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-3370" windowWidth="38620" windowHeight="21220" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
   <si>
     <t xml:space="preserve">Please include the proposals under your name </t>
   </si>
@@ -76,13 +76,24 @@
   </si>
   <si>
     <t>Question</t>
+  </si>
+  <si>
+    <t>Most effective workout based on BMI Category: We can calculate BMI and segment the dataset into four categories (Underweight, Normal, Overweight, Obese)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare average heart rate across different workout types (Cycling, Cardio, Strength, Yoga) [ANOVA] </t>
+  </si>
+  <si>
+    <t>Anomaly detection (Identify health risks):
+a.	Resting heart rate that's consistently above 100 bpm or below 60 bpm could indicate a problem.
+b.	Unusual spikes or dips in heart rate during workouts.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -483,25 +494,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2B683-EEB2-4C59-A502-E3C117712EB0}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.75" customWidth="1"/>
-    <col min="2" max="2" width="34.58203125" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="54.44140625" customWidth="1"/>
     <col min="5" max="5" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
@@ -510,7 +521,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -533,17 +544,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="56">
+    <row r="7" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
@@ -551,7 +562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="56">
+    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>3</v>
       </c>
@@ -559,7 +570,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="56">
+    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>3</v>
       </c>
@@ -567,7 +578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="70">
+    <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>3</v>
       </c>
@@ -576,14 +587,33 @@
       </c>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>5</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Update SMART Question Proposals.xlsx"
</commit_message>
<xml_diff>
--- a/midterm/SMART Question Proposals.xlsx
+++ b/midterm/SMART Question Proposals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/225622b72ce7f783/Documents/GWU/Semester 1/DATS 6101 - Introduction to Data Science/Mid Term Project/team_galileo/midterm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisgamo\Documents\GitHub\team_galileo\midterm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{FF3516DF-7292-4117-A3F4-32BC3B380EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6864B3C-B5B6-4B44-84E3-A2ADA305C908}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3516DF-7292-4117-A3F4-32BC3B380EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
+    <workbookView xWindow="-38510" yWindow="-3370" windowWidth="38620" windowHeight="21220" xr2:uid="{28466A7A-6B60-4074-A71F-EDDC329E068B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t xml:space="preserve">Please include the proposals under your name </t>
   </si>
@@ -76,24 +76,13 @@
   </si>
   <si>
     <t>Question</t>
-  </si>
-  <si>
-    <t>Most effective workout based on BMI Category: We can calculate BMI and segment the dataset into four categories (Underweight, Normal, Overweight, Obese)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compare average heart rate across different workout types (Cycling, Cardio, Strength, Yoga) [ANOVA] </t>
-  </si>
-  <si>
-    <t>Anomaly detection (Identify health risks):
-a.	Resting heart rate that's consistently above 100 bpm or below 60 bpm could indicate a problem.
-b.	Unusual spikes or dips in heart rate during workouts.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,25 +483,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2B683-EEB2-4C59-A502-E3C117712EB0}">
-  <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="2" width="54.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.75" customWidth="1"/>
+    <col min="2" max="2" width="34.58203125" customWidth="1"/>
     <col min="5" max="5" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
@@ -521,7 +510,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -544,17 +533,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="56">
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
@@ -562,7 +551,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="56">
       <c r="A8" s="5" t="s">
         <v>3</v>
       </c>
@@ -570,7 +559,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="56">
       <c r="A9" s="5" t="s">
         <v>3</v>
       </c>
@@ -578,7 +567,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="70">
       <c r="A10" s="5" t="s">
         <v>3</v>
       </c>
@@ -587,33 +576,14 @@
       </c>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
         <v>5</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>